<commit_message>
Dynamic capital design templates, year checks, and improved data handling
Year range validated and stored during model upload; mismatches prevent loading. Capital design and general info templates auto-adjust to model year range (2020–2050 baseline, trimmed by models).

LPG general info dynamically generates EBITDA and OPEX rows per model uploaded.

Empty capital design templates (equity/grants/debt) for each base tech (electricity, carbon, LPG) and dinamically adaptative to additional ones. Design tables with customizable heights per sheet to remove empty space.

Integrated save/reset buttons for each sheet, linked to backend endpoints. Subtables handled by splitting and reconstructing DataFrames based on header content.

Editable columns defined via per-subtable dictionaries for ag-grid integration.
</commit_message>
<xml_diff>
--- a/backend/general-information/general-information-template.xlsx
+++ b/backend/general-information/general-information-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8954da175e61d5af/Escritorio/IIT/NICCP-AI/backend/general-information/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="13_ncr:3_{297C9F4D-5BEC-4077-8986-513ACDF59508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3F835B8F-1126-42E4-AB73-154E1FF14EA4}"/>
+  <xr:revisionPtr revIDLastSave="64" documentId="13_ncr:3_{297C9F4D-5BEC-4077-8986-513ACDF59508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{081C4B09-E6B4-4C23-A980-2943EFEF6A50}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Electricity" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="47">
   <si>
     <t>Inputs</t>
   </si>
@@ -94,12 +94,6 @@
     <t>Trade payables - Days of OPEX costs</t>
   </si>
   <si>
-    <t>% EBITDA Margin - {model}</t>
-  </si>
-  <si>
-    <t>OPEX subsidies - {model}</t>
-  </si>
-  <si>
     <t>CO2 certificate (%) - from the total CO2 avoided</t>
   </si>
   <si>
@@ -167,6 +161,21 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>2020</t>
+  </si>
+  <si>
+    <t>2021</t>
+  </si>
+  <si>
+    <t>2022</t>
+  </si>
+  <si>
+    <t>2023</t>
+  </si>
+  <si>
+    <t>2024</t>
   </si>
 </sst>
 </file>
@@ -185,11 +194,13 @@
       <b/>
       <sz val="11"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
@@ -271,6 +282,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -590,10 +605,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AC5"/>
+  <dimension ref="A1:AH5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -604,85 +619,100 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="S1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="U1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="W1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="AA1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="AB1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="AC1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="AD1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="AE1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="AF1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="AG1" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AH1" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="AB1" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="AC1" s="2" t="s">
-        <v>42</v>
-      </c>
     </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -770,8 +800,23 @@
       <c r="AC2">
         <v>0</v>
       </c>
+      <c r="AD2">
+        <v>0</v>
+      </c>
+      <c r="AE2">
+        <v>0</v>
+      </c>
+      <c r="AF2">
+        <v>0</v>
+      </c>
+      <c r="AG2">
+        <v>0</v>
+      </c>
+      <c r="AH2">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -859,8 +904,23 @@
       <c r="AC3">
         <v>0</v>
       </c>
+      <c r="AD3">
+        <v>0</v>
+      </c>
+      <c r="AE3">
+        <v>0</v>
+      </c>
+      <c r="AF3">
+        <v>0</v>
+      </c>
+      <c r="AG3">
+        <v>0</v>
+      </c>
+      <c r="AH3">
+        <v>0</v>
+      </c>
     </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -948,8 +1008,23 @@
       <c r="AC4">
         <v>0</v>
       </c>
+      <c r="AD4">
+        <v>0</v>
+      </c>
+      <c r="AE4">
+        <v>0</v>
+      </c>
+      <c r="AF4">
+        <v>0</v>
+      </c>
+      <c r="AG4">
+        <v>0</v>
+      </c>
+      <c r="AH4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -1035,6 +1110,21 @@
         <v>0</v>
       </c>
       <c r="AC5">
+        <v>0</v>
+      </c>
+      <c r="AD5">
+        <v>0</v>
+      </c>
+      <c r="AE5">
+        <v>0</v>
+      </c>
+      <c r="AF5">
+        <v>0</v>
+      </c>
+      <c r="AG5">
+        <v>0</v>
+      </c>
+      <c r="AH5">
         <v>0</v>
       </c>
     </row>
@@ -1046,13 +1136,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AC7"/>
+  <dimension ref="A1:AH5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="31.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1063,85 +1153,100 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="S1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="U1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AB1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="AC1" s="1" t="s">
-        <v>42</v>
-      </c>
     </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -1229,8 +1334,23 @@
       <c r="AC2">
         <v>0</v>
       </c>
+      <c r="AD2">
+        <v>0</v>
+      </c>
+      <c r="AE2">
+        <v>0</v>
+      </c>
+      <c r="AF2">
+        <v>0</v>
+      </c>
+      <c r="AG2">
+        <v>0</v>
+      </c>
+      <c r="AH2">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1318,8 +1438,23 @@
       <c r="AC3">
         <v>0</v>
       </c>
+      <c r="AD3">
+        <v>0</v>
+      </c>
+      <c r="AE3">
+        <v>0</v>
+      </c>
+      <c r="AF3">
+        <v>0</v>
+      </c>
+      <c r="AG3">
+        <v>0</v>
+      </c>
+      <c r="AH3">
+        <v>0</v>
+      </c>
     </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1407,8 +1542,23 @@
       <c r="AC4">
         <v>0</v>
       </c>
+      <c r="AD4">
+        <v>0</v>
+      </c>
+      <c r="AE4">
+        <v>0</v>
+      </c>
+      <c r="AF4">
+        <v>0</v>
+      </c>
+      <c r="AG4">
+        <v>0</v>
+      </c>
+      <c r="AH4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -1496,182 +1646,19 @@
       <c r="AC5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-      <c r="D6">
-        <v>0</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6">
-        <v>0</v>
-      </c>
-      <c r="G6">
-        <v>0</v>
-      </c>
-      <c r="H6">
-        <v>0</v>
-      </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
-      <c r="J6">
-        <v>0</v>
-      </c>
-      <c r="K6">
-        <v>0</v>
-      </c>
-      <c r="L6">
-        <v>0</v>
-      </c>
-      <c r="M6">
-        <v>0</v>
-      </c>
-      <c r="N6">
-        <v>0</v>
-      </c>
-      <c r="O6">
-        <v>0</v>
-      </c>
-      <c r="P6">
-        <v>0</v>
-      </c>
-      <c r="Q6">
-        <v>0</v>
-      </c>
-      <c r="R6">
-        <v>0</v>
-      </c>
-      <c r="S6">
-        <v>0</v>
-      </c>
-      <c r="T6">
-        <v>0</v>
-      </c>
-      <c r="U6">
-        <v>0</v>
-      </c>
-      <c r="V6">
-        <v>0</v>
-      </c>
-      <c r="W6">
-        <v>0</v>
-      </c>
-      <c r="X6">
-        <v>0</v>
-      </c>
-      <c r="Y6">
-        <v>0</v>
-      </c>
-      <c r="Z6">
-        <v>0</v>
-      </c>
-      <c r="AA6">
-        <v>0</v>
-      </c>
-      <c r="AB6">
-        <v>0</v>
-      </c>
-      <c r="AC6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7">
-        <v>0</v>
-      </c>
-      <c r="H7">
-        <v>0</v>
-      </c>
-      <c r="I7">
-        <v>0</v>
-      </c>
-      <c r="J7">
-        <v>0</v>
-      </c>
-      <c r="K7">
-        <v>0</v>
-      </c>
-      <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="M7">
-        <v>0</v>
-      </c>
-      <c r="N7">
-        <v>0</v>
-      </c>
-      <c r="O7">
-        <v>0</v>
-      </c>
-      <c r="P7">
-        <v>0</v>
-      </c>
-      <c r="Q7">
-        <v>0</v>
-      </c>
-      <c r="R7">
-        <v>0</v>
-      </c>
-      <c r="S7">
-        <v>0</v>
-      </c>
-      <c r="T7">
-        <v>0</v>
-      </c>
-      <c r="U7">
-        <v>0</v>
-      </c>
-      <c r="V7">
-        <v>0</v>
-      </c>
-      <c r="W7">
-        <v>0</v>
-      </c>
-      <c r="X7">
-        <v>0</v>
-      </c>
-      <c r="Y7">
-        <v>0</v>
-      </c>
-      <c r="Z7">
-        <v>0</v>
-      </c>
-      <c r="AA7">
-        <v>0</v>
-      </c>
-      <c r="AB7">
-        <v>0</v>
-      </c>
-      <c r="AC7">
+      <c r="AD5">
+        <v>0</v>
+      </c>
+      <c r="AE5">
+        <v>0</v>
+      </c>
+      <c r="AF5">
+        <v>0</v>
+      </c>
+      <c r="AG5">
+        <v>0</v>
+      </c>
+      <c r="AH5">
         <v>0</v>
       </c>
     </row>
@@ -1683,13 +1670,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{916D2B2D-4AA6-4AEC-A74D-5F74F284844E}">
-  <dimension ref="A1:AC5"/>
+  <dimension ref="A1:AH5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="31.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1700,87 +1687,102 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="S1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="U1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AB1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="AC1" s="1" t="s">
-        <v>42</v>
-      </c>
     </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B2" t="s">
         <v>14</v>
@@ -1866,10 +1868,25 @@
       <c r="AC2">
         <v>0</v>
       </c>
+      <c r="AD2">
+        <v>0</v>
+      </c>
+      <c r="AE2">
+        <v>0</v>
+      </c>
+      <c r="AF2">
+        <v>0</v>
+      </c>
+      <c r="AG2">
+        <v>0</v>
+      </c>
+      <c r="AH2">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s">
         <v>14</v>
@@ -1955,186 +1972,232 @@
       <c r="AC3">
         <v>0</v>
       </c>
+      <c r="AD3">
+        <v>0</v>
+      </c>
+      <c r="AE3">
+        <v>0</v>
+      </c>
+      <c r="AF3">
+        <v>0</v>
+      </c>
+      <c r="AG3">
+        <v>0</v>
+      </c>
+      <c r="AH3">
+        <v>0</v>
+      </c>
     </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>0</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <v>0</v>
+      </c>
+      <c r="U4">
+        <v>0</v>
+      </c>
+      <c r="V4">
+        <v>0</v>
+      </c>
+      <c r="W4">
+        <v>0</v>
+      </c>
+      <c r="X4">
+        <v>0</v>
+      </c>
+      <c r="Y4">
+        <v>0</v>
+      </c>
+      <c r="Z4">
+        <v>0</v>
+      </c>
+      <c r="AA4">
+        <v>0</v>
+      </c>
+      <c r="AB4">
+        <v>0</v>
+      </c>
+      <c r="AC4">
+        <v>0</v>
+      </c>
+      <c r="AD4">
+        <v>0</v>
+      </c>
+      <c r="AE4">
+        <v>0</v>
+      </c>
+      <c r="AF4">
+        <v>0</v>
+      </c>
+      <c r="AG4">
+        <v>0</v>
+      </c>
+      <c r="AH4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>23</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
         <v>24</v>
       </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4">
-        <v>0</v>
-      </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
-      <c r="L4">
-        <v>0</v>
-      </c>
-      <c r="M4">
-        <v>0</v>
-      </c>
-      <c r="N4">
-        <v>0</v>
-      </c>
-      <c r="O4">
-        <v>0</v>
-      </c>
-      <c r="P4">
-        <v>0</v>
-      </c>
-      <c r="Q4">
-        <v>0</v>
-      </c>
-      <c r="R4">
-        <v>0</v>
-      </c>
-      <c r="S4">
-        <v>0</v>
-      </c>
-      <c r="T4">
-        <v>0</v>
-      </c>
-      <c r="U4">
-        <v>0</v>
-      </c>
-      <c r="V4">
-        <v>0</v>
-      </c>
-      <c r="W4">
-        <v>0</v>
-      </c>
-      <c r="X4">
-        <v>0</v>
-      </c>
-      <c r="Y4">
-        <v>0</v>
-      </c>
-      <c r="Z4">
-        <v>0</v>
-      </c>
-      <c r="AA4">
-        <v>0</v>
-      </c>
-      <c r="AB4">
-        <v>0</v>
-      </c>
-      <c r="AC4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" t="s">
-        <v>26</v>
-      </c>
       <c r="C5">
         <v>0</v>
       </c>
       <c r="D5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="G5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="H5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="I5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="J5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="K5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="L5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="M5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="N5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="P5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Q5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="R5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="S5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="T5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="U5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="V5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="W5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="X5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Y5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Z5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="AA5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="AB5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="AC5" t="s">
-        <v>43</v>
+        <v>41</v>
+      </c>
+      <c r="AD5" t="s">
+        <v>41</v>
+      </c>
+      <c r="AE5" t="s">
+        <v>41</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>41</v>
+      </c>
+      <c r="AG5" t="s">
+        <v>41</v>
+      </c>
+      <c r="AH5" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>